<commit_message>
Changes in accounts section
</commit_message>
<xml_diff>
--- a/AlNoor_ERP_Dataset.xlsx
+++ b/AlNoor_ERP_Dataset.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Desktop\Fyp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{784883B3-AF99-43B5-8029-D8806B24D077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3282FCA-5FE6-41F5-A004-4F7B4E9BF694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="300" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <sheet name="Employees" sheetId="7" r:id="rId9"/>
     <sheet name="Summary Dashboard" sheetId="8" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>

</xml_diff>